<commit_message>
Sort recommendations best-first everywhere + Google Sheets clean-reuse
- Sort the source `live` once by strength tier (STRONG BUY->BUY->ACCUMULATE->
  WATCH) then Evidence Score desc then weight. xlsx, canonical CSV, Telegram and
  Google Sheets all inherit the same top-to-bottom order (best at top).
- sheets_sync --clean: write the 8 AEGIS tabs then remove leftover tabs, so an
  existing spreadsheet can be reused entirely for AEGIS (no rename).

Verified: Telegram + AEGIS_LATEST.xlsx + Google Sheet all show identical sorted order.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/AEGIS_LATEST.xlsx
+++ b/reports/AEGIS_LATEST.xlsx
@@ -1275,39 +1275,39 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C2" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>88</v>
       </c>
       <c r="E2" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="F2" t="n">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="G2" t="n">
         <v>60</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>25570</v>
+        <v>8457</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>24850 - 26290</t>
+          <t>8242 - 8672</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -1321,15 +1321,15 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-8.6%)</t>
+          <t>Above 200-DMA (+11.2%)</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -1342,22 +1342,22 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>25570</v>
+        <v>25371</v>
       </c>
       <c r="T2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U2" t="n">
-        <v>11.3</v>
+        <v>10.9</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ABBOTINDIA: 65; TORNTPHARM: 78, CIPLA: 73, ZYDUSLIFE: 72. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — APOLLOHOSP: 80; FORTIS: 72, MAXHEALTH: 70, METROPOLIS: 64</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Low-risk Pharma holding (low vol) • below 200-dma (-8.6%) • sector strength 65/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +24.6%</t>
+          <t>Low-risk Healthcare holding (low vol) • above 200-dma (+11.2%) • outperforming Nifty • sector strength 94/100 • regime cautious (partial deploy) • 4 similar past recs: 75% positive, median +5.9%</t>
         </is>
       </c>
     </row>
@@ -1368,39 +1368,39 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="D3" t="n">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E3" t="n">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="F3" t="n">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="G3" t="n">
         <v>60</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>2357.8</v>
+        <v>364.6</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2298 - 2418</t>
+          <t>354 - 375</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1414,15 +1414,15 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+9.3%)</t>
+          <t>Above 200-DMA (+2.7%)</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -1435,22 +1435,22 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>33009</v>
+        <v>17136</v>
       </c>
       <c r="T3" t="n">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="U3" t="n">
-        <v>11</v>
+        <v>5.8</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — LUPIN: 71; TORNTPHARM: 78, CIPLA: 73, ZYDUSLIFE: 72. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — NTPC: 80; POWERGRID: 72, TATAPOWER: 68, CESC: 62</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Low-risk Pharma holding (low vol) • above 200-dma (+9.3%) • sector strength 65/100 • regime cautious (partial deploy) • no historical analogue yet (&lt;3 obs)</t>
+          <t>Low-risk Power holding (low vol) • above 200-dma (+2.7%) • sector strength 88/100 • regime cautious (partial deploy) • 4 similar past recs: 100% positive, median +11.5%</t>
         </is>
       </c>
     </row>
@@ -1461,39 +1461,39 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C4" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D4" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="G4" t="n">
         <v>60</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>8457</v>
+        <v>821</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>8242 - 8672</t>
+          <t>801 - 841</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1507,15 +1507,15 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+11.2%)</t>
+          <t>Above 200-DMA (+8.5%)</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -1528,22 +1528,22 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>25371</v>
+        <v>27095</v>
       </c>
       <c r="T4" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="U4" t="n">
-        <v>10.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — APOLLOHOSP: 80; FORTIS: 72, MAXHEALTH: 70, METROPOLIS: 64</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — MARICO: 72; NESTLEIND: 74, VBL: 58, TATACONSUM: 56. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Low-risk Healthcare holding (low vol) • above 200-dma (+11.2%) • outperforming Nifty • sector strength 94/100 • regime cautious (partial deploy) • 4 similar past recs: 75% positive, median +5.9%</t>
+          <t>Low-risk FMCG holding (low vol) • above 200-dma (+8.5%) • sector strength 29/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +3.3%</t>
         </is>
       </c>
     </row>
@@ -1554,61 +1554,61 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C5" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="D5" t="n">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E5" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="F5" t="n">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="G5" t="n">
         <v>60</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1901.6</v>
+        <v>291.9</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1851 - 1952</t>
+          <t>283 - 301</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>-3% to +15%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-2.6%)</t>
+          <t>Above 200-DMA (+2.1%)</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -1621,65 +1621,65 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>30426</v>
+        <v>16349</v>
       </c>
       <c r="T5" t="n">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="U5" t="n">
-        <v>10.2</v>
+        <v>5.5</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BHARTIARTL: 70; TATACOMM: 54, INDUSTOWER: 52</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — POWERGRID: 72; NTPC: 80, TATAPOWER: 68, CESC: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Low-risk Telecom holding (low vol) • below 200-dma (-2.6%) • sector strength 59/100 • regime cautious (partial deploy) • 13 similar past recs: 69% positive, median +12.5%</t>
+          <t>Low-risk Power holding (low vol) • above 200-dma (+2.1%) • sector strength 88/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +12.3%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>WATCH</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="C6" t="n">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="D6" t="n">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="E6" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F6" t="n">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="G6" t="n">
         <v>60</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>5241</v>
+        <v>2357.8</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>5103 - 5379</t>
+          <t>2298 - 2418</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1693,11 +1693,11 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-9.6%)</t>
+          <t>Above 200-DMA (+9.3%)</t>
         </is>
       </c>
       <c r="P6" t="n">
@@ -1714,22 +1714,22 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>26205</v>
+        <v>33009</v>
       </c>
       <c r="T6" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="U6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BRITANNIA: 51; NESTLEIND: 74, MARICO: 72, VBL: 58. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — LUPIN: 71; TORNTPHARM: 78, CIPLA: 73, ZYDUSLIFE: 72. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Low-risk FMCG holding (low vol) • below 200-dma (-9.6%) • sector strength 29/100 • regime cautious (partial deploy) • 3 similar past recs: 33% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
+          <t>Low-risk Pharma holding (low vol) • above 200-dma (+9.3%) • sector strength 65/100 • regime cautious (partial deploy) • no historical analogue yet (&lt;3 obs)</t>
         </is>
       </c>
     </row>
@@ -1740,61 +1740,61 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C7" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="D7" t="n">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F7" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="G7" t="n">
         <v>60</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Telecom</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>821</v>
+        <v>1901.6</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>801 - 841</t>
+          <t>1851 - 1952</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-3% to +15%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+8.5%)</t>
+          <t>Below 200-DMA (-2.6%)</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1807,87 +1807,87 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>27095</v>
+        <v>30426</v>
       </c>
       <c r="T7" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="U7" t="n">
-        <v>9.199999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — MARICO: 72; NESTLEIND: 74, VBL: 58, TATACONSUM: 56. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BHARTIARTL: 70; TATACOMM: 54, INDUSTOWER: 52</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Low-risk FMCG holding (low vol) • above 200-dma (+8.5%) • sector strength 29/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +3.3%</t>
+          <t>Low-risk Telecom holding (low vol) • below 200-dma (-2.6%) • sector strength 59/100 • regime cautious (partial deploy) • 13 similar past recs: 69% positive, median +12.5%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C8" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="D8" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E8" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F8" t="n">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="G8" t="n">
         <v>60</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>ABBOTINDIA</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="J8" t="n">
-        <v>1309.5</v>
+        <v>25570</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1268 - 1351</t>
+          <t>24850 - 26290</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>-1% to +7%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-7.8%)</t>
+          <t>Below 200-DMA (-8.6%)</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1900,22 +1900,22 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>22262</v>
+        <v>25570</v>
       </c>
       <c r="T8" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>7.7</v>
+        <v>11.3</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — RELIANCE: 55; GAIL: 60, IGL: 52, PETRONET: 49. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ABBOTINDIA: 65; TORNTPHARM: 78, CIPLA: 73, ZYDUSLIFE: 72. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>Low-risk Energy holding (low vol) • below 200-dma (-7.8%) • sector strength 18/100 • regime cautious (partial deploy) • 8 similar past recs: 62% positive, median +4.3%</t>
+          <t>Low-risk Pharma holding (low vol) • below 200-dma (-8.6%) • sector strength 65/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +24.6%</t>
         </is>
       </c>
     </row>
@@ -1926,16 +1926,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C9" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="D9" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E9" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F9" t="n">
         <v>35</v>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1954,33 +1954,33 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>1833.7</v>
+        <v>1338.3</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1782 - 1885</t>
+          <t>1300 - 1377</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+2% to +8%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-2.5%)</t>
+          <t>Below 200-DMA (-0.6%)</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1993,22 +1993,22 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>20171</v>
+        <v>17398</v>
       </c>
       <c r="T9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="U9" t="n">
-        <v>7.1</v>
+        <v>5.9</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIGI: 59; AXISBANK: 62, ICICIBANK: 62, KOTAKBANK: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIBANK: 62; AXISBANK: 62, KOTAKBANK: 62, LICI: 62</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Low-risk Financials holding (low vol) • below 200-dma (-2.5%) • sector strength 35/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +7.7%</t>
+          <t>Low-risk Financials holding (low vol) • below 200-dma (-0.6%) • sector strength 35/100 • regime cautious (partial deploy) • 8 similar past recs: 75% positive, median +5.3%</t>
         </is>
       </c>
     </row>
@@ -2019,16 +2019,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C10" t="n">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D10" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E10" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F10" t="n">
         <v>35</v>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>ICICIGI</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2047,33 +2047,33 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1338.3</v>
+        <v>1833.7</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1300 - 1377</t>
+          <t>1782 - 1885</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>+2% to +8%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N10" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-0.6%)</t>
+          <t>Below 200-DMA (-2.5%)</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -2086,87 +2086,87 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>17398</v>
+        <v>20171</v>
       </c>
       <c r="T10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="U10" t="n">
-        <v>5.9</v>
+        <v>7.1</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIBANK: 62; AXISBANK: 62, KOTAKBANK: 62, LICI: 62</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIGI: 59; AXISBANK: 62, ICICIBANK: 62, KOTAKBANK: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>Low-risk Financials holding (low vol) • below 200-dma (-0.6%) • sector strength 35/100 • regime cautious (partial deploy) • 8 similar past recs: 75% positive, median +5.3%</t>
+          <t>Low-risk Financials holding (low vol) • below 200-dma (-2.5%) • sector strength 35/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +7.7%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>BUY</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C11" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="D11" t="n">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="E11" t="n">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F11" t="n">
-        <v>88</v>
+        <v>18</v>
       </c>
       <c r="G11" t="n">
         <v>60</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>364.6</v>
+        <v>1309.5</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>354 - 375</t>
+          <t>1268 - 1351</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-1% to +7%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>62%</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+2.7%)</t>
+          <t>Below 200-DMA (-7.8%)</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -2179,65 +2179,65 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>17136</v>
+        <v>22262</v>
       </c>
       <c r="T11" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="U11" t="n">
-        <v>5.8</v>
+        <v>7.7</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — NTPC: 80; POWERGRID: 72, TATAPOWER: 68, CESC: 62</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — RELIANCE: 55; GAIL: 60, IGL: 52, PETRONET: 49. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Low-risk Power holding (low vol) • above 200-dma (+2.7%) • sector strength 88/100 • regime cautious (partial deploy) • 4 similar past recs: 100% positive, median +11.5%</t>
+          <t>Low-risk Energy holding (low vol) • below 200-dma (-7.8%) • sector strength 18/100 • regime cautious (partial deploy) • 8 similar past recs: 62% positive, median +4.3%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>STRONG BUY</t>
+          <t>WATCH</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>72</v>
+        <v>51</v>
       </c>
       <c r="C12" t="n">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="D12" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="E12" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="F12" t="n">
-        <v>88</v>
+        <v>29</v>
       </c>
       <c r="G12" t="n">
         <v>60</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>291.9</v>
+        <v>5241</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>283 - 301</t>
+          <t>5103 - 5379</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2251,15 +2251,15 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+2.1%)</t>
+          <t>Below 200-DMA (-9.6%)</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -2272,22 +2272,22 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>16349</v>
+        <v>26205</v>
       </c>
       <c r="T12" t="n">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="U12" t="n">
-        <v>5.5</v>
+        <v>10</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — POWERGRID: 72; NTPC: 80, TATAPOWER: 68, CESC: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BRITANNIA: 51; NESTLEIND: 74, MARICO: 72, VBL: 58. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>Low-risk Power holding (low vol) • above 200-dma (+2.1%) • sector strength 88/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +12.3%</t>
+          <t>Low-risk FMCG holding (low vol) • below 200-dma (-9.6%) • sector strength 29/100 • regime cautious (partial deploy) • 3 similar past recs: 33% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.3 explainability: score decomposition + recommendation attribution
Pure explainability of the EXISTING model (no new scoring), per the reviewer:

- SCORE DECOMPOSITION: the Overall score is shown as its exact weighted parts,
  e.g. APOLLOHOSP "Risk/Vol +25 · Historical +19 · Trend/Tech +16 · Regime +9 ·
  Sector +9 = 78". They sum to the total — nothing invented. Makes the engine
  debuggable and honestly shows Risk/Vol is the dominant driver (it IS a risk engine).

- RECOMMENDATION ATTRIBUTION: per pick — Top Factor, Weakest Factor, "Selected
  Because" (strongest factors + the lowest-vol/sector-cap rule), and an explicit
  "Not Evaluated: Fundamentals · Earnings · News · Flows" so the missing
  information is stated, not hidden.

Surfaced as columns in Today's Recommendations (workbook + Google Sheet).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/AEGIS_LATEST.xlsx
+++ b/reports/AEGIS_LATEST.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>APOLLOHOSP (score 77)</t>
+          <t>APOLLOHOSP (score 78)</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SHREECEM (score 49)</t>
+          <t>SHREECEM (score 48)</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:AB13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1389,105 +1389,130 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Score Breakdown</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Top Factor</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Weakest Factor</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>F: Historical</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>F: Technical/Trend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>F: Risk/Vol</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>F: Sector</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>F: Regime</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Stock</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Current Price</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Buy Range</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Expected Range (hist)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Prob +ve</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Rec Confidence %</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Trend</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Recommended Holding</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Review Date</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Allocation Rs</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Weight %</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Selected Because</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Why This vs Alternatives</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
@@ -1500,87 +1525,112 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
-      </c>
-      <c r="C2" t="n">
+        <v>78</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Risk/Vol +25 · Historical +19 · Trend/Tech +16 · Regime +9 · Sector +9 = 78</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>64</v>
       </c>
-      <c r="D2" t="n">
+      <c r="G2" t="n">
         <v>78</v>
       </c>
-      <c r="E2" t="n">
+      <c r="H2" t="n">
         <v>99</v>
       </c>
-      <c r="F2" t="n">
+      <c r="I2" t="n">
         <v>88</v>
       </c>
-      <c r="G2" t="n">
+      <c r="J2" t="n">
         <v>60</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>APOLLOHOSP</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="M2" t="n">
         <v>8592</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>8374 - 8810</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="Q2" t="n">
         <v>78</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Above 200-DMA (+12.8%)</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="S2" t="n">
         <v>71</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="V2" t="n">
         <v>25776</v>
       </c>
-      <c r="T2" t="n">
+      <c r="W2" t="n">
         <v>3</v>
       </c>
-      <c r="U2" t="n">
+      <c r="X2" t="n">
         <v>9</v>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — APOLLOHOSP: 77; FORTIS: 71, MAXHEALTH: 69, LALPATHLAB: 61</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Healthcare name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — APOLLOHOSP: 78; FORTIS: 70, MAXHEALTH: 69, LALPATHLAB: 61</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Low-risk Healthcare holding (low vol) • above 200-dma (+12.8%) • outperforming Nifty • sector strength 88/100 • regime cautious (partial deploy) • 4 similar past recs: 75% positive, median +5.9%</t>
         </is>
@@ -1595,85 +1645,110 @@
       <c r="B3" t="n">
         <v>72</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Risk/Vol +25 · Historical +18 · Trend/Tech +17 · Regime +9 · Sector +3 = 72</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>61</v>
       </c>
-      <c r="D3" t="n">
+      <c r="G3" t="n">
         <v>84</v>
       </c>
-      <c r="E3" t="n">
+      <c r="H3" t="n">
         <v>100</v>
       </c>
-      <c r="F3" t="n">
+      <c r="I3" t="n">
         <v>29</v>
       </c>
-      <c r="G3" t="n">
+      <c r="J3" t="n">
         <v>60</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>MARICO</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="M3" t="n">
         <v>825.8</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>806 - 846</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="Q3" t="n">
         <v>75</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Above 200-DMA (+9.0%)</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="S3" t="n">
         <v>59</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="V3" t="n">
         <v>23948</v>
       </c>
-      <c r="T3" t="n">
+      <c r="W3" t="n">
         <v>29</v>
       </c>
-      <c r="U3" t="n">
+      <c r="X3" t="n">
         <v>8.1</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility FMCG name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — MARICO: 72; NESTLEIND: 73, VBL: 61, UNITDSPR: 60. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>Low-risk FMCG holding (low vol) • above 200-dma (+9.0%) • sector strength 29/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +3.3%</t>
         </is>
@@ -1686,89 +1761,114 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
-      </c>
-      <c r="C4" t="n">
-        <v>84</v>
-      </c>
-      <c r="D4" t="n">
-        <v>24</v>
-      </c>
-      <c r="E4" t="n">
-        <v>93</v>
+        <v>71</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Risk/Vol +24 · Historical +19 · Trend/Tech +15 · Regime +9 · Sector +4 = 71</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
       </c>
       <c r="F4" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="G4" t="n">
+        <v>75</v>
+      </c>
+      <c r="H4" t="n">
+        <v>94</v>
+      </c>
+      <c r="I4" t="n">
+        <v>35</v>
+      </c>
+      <c r="J4" t="n">
         <v>60</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Power</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>352</v>
-      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>342 - 363</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>409</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>397 - 421</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N4" t="n">
-        <v>74</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Below 200-DMA (-0.9%)</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" t="n">
+        <v>75</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Above 200-DMA (+0.7%)</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>81</v>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S4" t="n">
-        <v>23235</v>
-      </c>
-      <c r="T4" t="n">
-        <v>66</v>
-      </c>
-      <c r="U4" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — NTPC: 70; POWERGRID: 62, CESC: 60, NHPC: 59</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>Low-risk Power holding (low vol) • below 200-dma (-0.9%) • sector strength 76/100 • regime cautious (partial deploy) • 4 similar past recs: 100% positive, median +11.5%</t>
+      <c r="V4" t="n">
+        <v>17996</v>
+      </c>
+      <c r="W4" t="n">
+        <v>44</v>
+      </c>
+      <c r="X4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Financials name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — KOTAKBANK: 71; ICICIBANK: 72, AXISBANK: 62, SBIN: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>Low-risk Financials holding (low vol) • above 200-dma (+0.7%) • outperforming Nifty • sector strength 35/100 • regime cautious (partial deploy) • 3 similar past recs: 100% positive, median +1.9%</t>
         </is>
       </c>
     </row>
@@ -1781,87 +1881,112 @@
       <c r="B5" t="n">
         <v>70</v>
       </c>
-      <c r="C5" t="n">
-        <v>64</v>
-      </c>
-      <c r="D5" t="n">
-        <v>75</v>
-      </c>
-      <c r="E5" t="n">
-        <v>94</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Historical +25 · Risk/Vol +23 · Regime +9 · Sector +8 · Trend/Tech +5 = 70</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Historical</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Trend/Tech</t>
+        </is>
       </c>
       <c r="F5" t="n">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="G5" t="n">
+        <v>24</v>
+      </c>
+      <c r="H5" t="n">
+        <v>93</v>
+      </c>
+      <c r="I5" t="n">
+        <v>76</v>
+      </c>
+      <c r="J5" t="n">
         <v>60</v>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>KOTAKBANK</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>409</v>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>397 - 421</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>352</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>342 - 363</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="Q5" t="n">
         <v>74</v>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Above 200-DMA (+0.7%)</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>81</v>
-      </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Below 200-DMA (-0.9%)</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>41</v>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S5" t="n">
-        <v>17996</v>
-      </c>
-      <c r="T5" t="n">
-        <v>44</v>
-      </c>
-      <c r="U5" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — KOTAKBANK: 70; ICICIBANK: 71, AXISBANK: 62, FEDERALBNK: 61. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Low-risk Financials holding (low vol) • above 200-dma (+0.7%) • outperforming Nifty • sector strength 35/100 • regime cautious (partial deploy) • 3 similar past recs: 100% positive, median +1.9%</t>
+      <c r="V5" t="n">
+        <v>23235</v>
+      </c>
+      <c r="W5" t="n">
+        <v>66</v>
+      </c>
+      <c r="X5" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Historical + Risk/Vol strongest; chosen as a lowest-volatility Power name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — NTPC: 70; POWERGRID: 62, CESC: 61, NHPC: 60</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>Low-risk Power holding (low vol) • below 200-dma (-0.9%) • sector strength 76/100 • regime cautious (partial deploy) • 4 similar past recs: 100% positive, median +11.5%</t>
         </is>
       </c>
     </row>
@@ -1872,87 +1997,112 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>68</v>
-      </c>
-      <c r="C6" t="n">
+        <v>69</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Risk/Vol +25 · Historical +15 · Trend/Tech +15 · Regime +9 · Sector +5 = 69</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>50</v>
       </c>
-      <c r="D6" t="n">
+      <c r="G6" t="n">
         <v>73</v>
       </c>
-      <c r="E6" t="n">
+      <c r="H6" t="n">
         <v>99</v>
       </c>
-      <c r="F6" t="n">
+      <c r="I6" t="n">
         <v>47</v>
       </c>
-      <c r="G6" t="n">
+      <c r="J6" t="n">
         <v>60</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>LUPIN</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Pharma</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="M6" t="n">
         <v>2343.5</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>2284 - 2403</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N6" t="n">
+      <c r="Q6" t="n">
         <v>71</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Above 200-DMA (+8.4%)</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="S6" t="n">
         <v>65</v>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S6" t="n">
+      <c r="V6" t="n">
         <v>35152</v>
       </c>
-      <c r="T6" t="n">
+      <c r="W6" t="n">
         <v>15</v>
       </c>
-      <c r="U6" t="n">
+      <c r="X6" t="n">
         <v>12.2</v>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — LUPIN: 68; TORNTPHARM: 76, CIPLA: 71, ZYDUSLIFE: 70. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Pharma name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — LUPIN: 69; TORNTPHARM: 77, CIPLA: 71, ZYDUSLIFE: 71. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
         <is>
           <t>Low-risk Pharma holding (low vol) • above 200-dma (+8.4%) • sector strength 47/100 • regime cautious (partial deploy) • no historical analogue yet (&lt;3 obs)</t>
         </is>
@@ -1965,87 +2115,112 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>67</v>
-      </c>
-      <c r="C7" t="n">
+        <v>66</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Risk/Vol +24 · Historical +23 · Regime +9 · Trend/Tech +6 · Sector +4 = 66</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>76</v>
       </c>
-      <c r="D7" t="n">
+      <c r="G7" t="n">
         <v>32</v>
       </c>
-      <c r="E7" t="n">
+      <c r="H7" t="n">
         <v>98</v>
       </c>
-      <c r="F7" t="n">
+      <c r="I7" t="n">
         <v>41</v>
       </c>
-      <c r="G7" t="n">
+      <c r="J7" t="n">
         <v>60</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>BHARTIARTL</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Telecom</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="M7" t="n">
         <v>1850.7</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>1801 - 1900</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>-3% to +15%</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>69%</t>
         </is>
       </c>
-      <c r="N7" t="n">
+      <c r="Q7" t="n">
         <v>85</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Below 200-DMA (-5.2%)</t>
         </is>
       </c>
-      <c r="P7" t="n">
+      <c r="S7" t="n">
         <v>60</v>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S7" t="n">
+      <c r="V7" t="n">
         <v>20358</v>
       </c>
-      <c r="T7" t="n">
+      <c r="W7" t="n">
         <v>11</v>
       </c>
-      <c r="U7" t="n">
+      <c r="X7" t="n">
         <v>7.1</v>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BHARTIARTL: 67; TATACOMM: 52, INDUSTOWER: 50</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Telecom name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BHARTIARTL: 66; TATACOMM: 53, INDUSTOWER: 50</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
         <is>
           <t>Low-risk Telecom holding (low vol) • below 200-dma (-5.2%) • sector strength 41/100 • regime cautious (partial deploy) • 13 similar past recs: 69% positive, median +12.5%</t>
         </is>
@@ -2060,85 +2235,110 @@
       <c r="B8" t="n">
         <v>64</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Risk/Vol +24 · Historical +21 · Regime +9 · Trend/Tech +5 · Sector +5 = 64</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
         <v>70</v>
       </c>
-      <c r="D8" t="n">
+      <c r="G8" t="n">
         <v>27</v>
       </c>
-      <c r="E8" t="n">
+      <c r="H8" t="n">
         <v>97</v>
       </c>
-      <c r="F8" t="n">
+      <c r="I8" t="n">
         <v>47</v>
       </c>
-      <c r="G8" t="n">
+      <c r="J8" t="n">
         <v>60</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>ABBOTINDIA</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Pharma</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="M8" t="n">
         <v>25585</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>24868 - 26302</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N8" t="n">
+      <c r="Q8" t="n">
         <v>72</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Below 200-DMA (-8.3%)</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="S8" t="n">
         <v>42</v>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S8" t="n">
+      <c r="V8" t="n">
         <v>25585</v>
       </c>
-      <c r="T8" t="n">
+      <c r="W8" t="n">
         <v>1</v>
       </c>
-      <c r="U8" t="n">
+      <c r="X8" t="n">
         <v>11.6</v>
       </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ABBOTINDIA: 64; TORNTPHARM: 76, CIPLA: 71, ZYDUSLIFE: 70. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Pharma name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ABBOTINDIA: 64; TORNTPHARM: 77, CIPLA: 71, ZYDUSLIFE: 71. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
         <is>
           <t>Low-risk Pharma holding (low vol) • below 200-dma (-8.3%) • sector strength 47/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +24.6%</t>
         </is>
@@ -2153,85 +2353,110 @@
       <c r="B9" t="n">
         <v>62</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Risk/Vol +23 · Historical +17 · Regime +9 · Sector +8 · Trend/Tech +5 = 62</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Trend/Tech</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
         <v>56</v>
       </c>
-      <c r="D9" t="n">
+      <c r="G9" t="n">
         <v>27</v>
       </c>
-      <c r="E9" t="n">
+      <c r="H9" t="n">
         <v>92</v>
       </c>
-      <c r="F9" t="n">
+      <c r="I9" t="n">
         <v>76</v>
       </c>
-      <c r="G9" t="n">
+      <c r="J9" t="n">
         <v>60</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>POWERGRID</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="M9" t="n">
         <v>283.9</v>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>275 - 293</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N9" t="n">
+      <c r="Q9" t="n">
         <v>71</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>Below 200-DMA (-0.8%)</t>
         </is>
       </c>
-      <c r="P9" t="n">
+      <c r="S9" t="n">
         <v>47</v>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S9" t="n">
+      <c r="V9" t="n">
         <v>19305</v>
       </c>
-      <c r="T9" t="n">
+      <c r="W9" t="n">
         <v>68</v>
       </c>
-      <c r="U9" t="n">
+      <c r="X9" t="n">
         <v>6.5</v>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — POWERGRID: 62; NTPC: 70, CESC: 60, NHPC: 59. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Power name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — POWERGRID: 62; NTPC: 70, CESC: 61, NHPC: 60. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
         <is>
           <t>Low-risk Power holding (low vol) • below 200-dma (-0.8%) • sector strength 76/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +12.3%</t>
         </is>
@@ -2244,87 +2469,112 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>59</v>
-      </c>
-      <c r="C10" t="n">
+        <v>60</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Risk/Vol +24 · Historical +16 · Regime +9 · Trend/Tech +7 · Sector +4 = 60</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
         <v>52</v>
       </c>
-      <c r="D10" t="n">
+      <c r="G10" t="n">
         <v>34</v>
       </c>
-      <c r="E10" t="n">
+      <c r="H10" t="n">
         <v>96</v>
       </c>
-      <c r="F10" t="n">
+      <c r="I10" t="n">
         <v>35</v>
       </c>
-      <c r="G10" t="n">
+      <c r="J10" t="n">
         <v>60</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>ICICIGI</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Financials</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="M10" t="n">
         <v>1813.6</v>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>1763 - 1865</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N10" t="n">
+      <c r="Q10" t="n">
         <v>70</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Below 200-DMA (-3.6%)</t>
         </is>
       </c>
-      <c r="P10" t="n">
+      <c r="S10" t="n">
         <v>57</v>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S10" t="n">
+      <c r="V10" t="n">
         <v>27204</v>
       </c>
-      <c r="T10" t="n">
+      <c r="W10" t="n">
         <v>15</v>
       </c>
-      <c r="U10" t="n">
+      <c r="X10" t="n">
         <v>9.1</v>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIGI: 59; ICICIBANK: 71, KOTAKBANK: 70, AXISBANK: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Financials name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIGI: 60; ICICIBANK: 72, KOTAKBANK: 71, AXISBANK: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
         <is>
           <t>Low-risk Financials holding (low vol) • below 200-dma (-3.6%) • sector strength 35/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +7.7%</t>
         </is>
@@ -2339,85 +2589,110 @@
       <c r="B11" t="n">
         <v>54</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Risk/Vol +22 · Historical +17 · Regime +9 · Trend/Tech +5 · Sector +1 = 54</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
         <v>56</v>
       </c>
-      <c r="D11" t="n">
+      <c r="G11" t="n">
         <v>25</v>
       </c>
-      <c r="E11" t="n">
+      <c r="H11" t="n">
         <v>90</v>
       </c>
-      <c r="F11" t="n">
+      <c r="I11" t="n">
         <v>12</v>
       </c>
-      <c r="G11" t="n">
+      <c r="J11" t="n">
         <v>60</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>RELIANCE</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Energy</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="M11" t="n">
         <v>1318.1</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>1276 - 1360</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>-1% to +7%</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>62%</t>
         </is>
       </c>
-      <c r="N11" t="n">
+      <c r="Q11" t="n">
         <v>72</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>Below 200-DMA (-7.2%)</t>
         </is>
       </c>
-      <c r="P11" t="n">
+      <c r="S11" t="n">
         <v>57</v>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S11" t="n">
+      <c r="V11" t="n">
         <v>25044</v>
       </c>
-      <c r="T11" t="n">
+      <c r="W11" t="n">
         <v>19</v>
       </c>
-      <c r="U11" t="n">
+      <c r="X11" t="n">
         <v>8.4</v>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — RELIANCE: 54; GAIL: 60, IGL: 51, PETRONET: 51. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Energy name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — RELIANCE: 54; GAIL: 59, IGL: 51, PETRONET: 50. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
         <is>
           <t>Low-risk Energy holding (low vol) • below 200-dma (-7.2%) • sector strength 12/100 • regime cautious (partial deploy) • 8 similar past recs: 62% positive, median +4.3%</t>
         </is>
@@ -2432,85 +2707,110 @@
       <c r="B12" t="n">
         <v>51</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Risk/Vol +24 · Historical +10 · Regime +9 · Trend/Tech +5 · Sector +3 = 51</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
         <v>32</v>
       </c>
-      <c r="D12" t="n">
+      <c r="G12" t="n">
         <v>25</v>
       </c>
-      <c r="E12" t="n">
+      <c r="H12" t="n">
         <v>98</v>
       </c>
-      <c r="F12" t="n">
+      <c r="I12" t="n">
         <v>29</v>
       </c>
-      <c r="G12" t="n">
+      <c r="J12" t="n">
         <v>60</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>BRITANNIA</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>FMCG</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="M12" t="n">
         <v>5237</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>5099 - 5375</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N12" t="n">
+      <c r="Q12" t="n">
         <v>66</v>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="R12" t="inlineStr">
         <is>
           <t>Below 200-DMA (-9.6%)</t>
         </is>
       </c>
-      <c r="P12" t="n">
+      <c r="S12" t="n">
         <v>62</v>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S12" t="n">
+      <c r="V12" t="n">
         <v>15711</v>
       </c>
-      <c r="T12" t="n">
+      <c r="W12" t="n">
         <v>3</v>
       </c>
-      <c r="U12" t="n">
+      <c r="X12" t="n">
         <v>7</v>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility FMCG name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
         <is>
           <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BRITANNIA: 51; NESTLEIND: 73, MARICO: 72, VBL: 61. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="AB12" t="inlineStr">
         <is>
           <t>Low-risk FMCG holding (low vol) • below 200-dma (-9.6%) • sector strength 29/100 • regime cautious (partial deploy) • 3 similar past recs: 33% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
         </is>
@@ -2523,87 +2823,112 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>49</v>
-      </c>
-      <c r="C13" t="n">
+        <v>48</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Risk/Vol +22 · Regime +9 · Trend/Tech +8 · Historical +7 · Sector +2 = 48</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Risk/Vol</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
         <v>24</v>
       </c>
-      <c r="D13" t="n">
+      <c r="G13" t="n">
         <v>41</v>
       </c>
-      <c r="E13" t="n">
+      <c r="H13" t="n">
         <v>90</v>
       </c>
-      <c r="F13" t="n">
+      <c r="I13" t="n">
         <v>18</v>
       </c>
-      <c r="G13" t="n">
+      <c r="J13" t="n">
         <v>60</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>SHREECEM</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Cement</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="M13" t="n">
         <v>25735</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>24925 - 26545</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>-11% to +3%</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="N13" t="n">
+      <c r="Q13" t="n">
         <v>70</v>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>Below 200-DMA (-2.7%)</t>
         </is>
       </c>
-      <c r="P13" t="n">
+      <c r="S13" t="n">
         <v>67</v>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>2 months (2M)</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="S13" t="n">
+      <c r="V13" t="n">
         <v>0</v>
       </c>
-      <c r="T13" t="n">
+      <c r="W13" t="n">
         <v>0</v>
       </c>
-      <c r="U13" t="n">
+      <c r="X13" t="n">
         <v>7.1</v>
       </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — SHREECEM: 49; GRASIM: 75, ULTRACEMCO: 57, RAMCOCEM: 48. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
-        </is>
-      </c>
-      <c r="W13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Risk/Vol + Regime strongest; chosen as a lowest-volatility Cement name under the sector cap</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Fundamentals · Earnings · News · Flows</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — SHREECEM: 48; GRASIM: 75, ULTRACEMCO: 57, RAMCOCEM: 48. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
         <is>
           <t>Low-risk Cement holding (low vol) • below 200-dma (-2.7%) • sector strength 18/100 • regime cautious (partial deploy) • 5 similar past recs: 40% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
         </is>

</xml_diff>

<commit_message>
Honest rename: "Portfolio Suitability" (not "Score") + Production/Lab operating model
The score measures risk-FIT, not expected outperformance — its dominant part is
always Risk/Vol. Renamed the displayed "Overall Score"/"Score /100" -> "Portfolio
Suitability", "Score Breakdown" -> "Suitability Breakdown", Telegram "score" ->
"suitability", TODAY "highest conviction" -> "best risk-fit". Methodology states
plainly: AEGIS is a portfolio-allocation engine, not an alpha-discovery engine.

docs/PRODUCTION_AND_LAB.md: formalises the operating model the reviewer asked for —
Production "1.x Stable" (FROZEN) vs Research "LAB-NNN" (nothing auto-promotes); the
dataset promotion pipeline; acquisition order; where AI belongs; 80-90% effort on data.

No new version tag — production stays frozen at 1.x; this is a labeling-honesty fix.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/AEGIS_LATEST.xlsx
+++ b/reports/AEGIS_LATEST.xlsx
@@ -531,24 +531,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Highest conviction</t>
+          <t>Best risk-fit (suitability)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>APOLLOHOSP (score 78)</t>
+          <t>APOLLOHOSP (78)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Weakest holding</t>
+          <t>Weakest holding (suitability)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SHREECEM (score 48)</t>
+          <t>SHREECEM (48)</t>
         </is>
       </c>
     </row>
@@ -1384,12 +1384,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Score /100</t>
+          <t>Portfolio Suitability</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Score Breakdown</t>
+          <t>Suitability Breakdown</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -27972,12 +27972,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Factor breakdown (each 0-100)</t>
+          <t>Portfolio Suitability (0-100)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Every pick shows 5 sub-scores so you see WHY, not one opaque number: Historical (win rate + median, SHRUNK toward neutral when &lt;5 cases), Technical/Trend (200-DMA, relative strength, RSI), Risk/Vol (low volatility = high), Sector, Regime. Overall = 0.30 Historical + 0.25 Risk + 0.20 Technical + 0.10 Sector + 0.15 Regime.</t>
+          <t>HONEST NAMING: this score measures how well a stock FITS a risk-managed portfolio (risk-fit), NOT how likely it is to outperform. Its largest component is always Risk/Vol — AEGIS is a portfolio-allocation engine, not an alpha-discovery engine. Built from 5 sub-scores: Historical (win rate + median, shrunk toward neutral when &lt;5 cases), Technical/Trend (200-DMA, rel-strength, RSI), Risk/Vol (low volatility = high), Sector, Regime. Suitability = 0.30 Historical + 0.25 Risk + 0.20 Technical + 0.10 Sector + 0.15 Regime (the Score Breakdown column shows the exact additive parts).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AEGIS run 2026-06-29: append data + refresh report + DB (manual local run)
</commit_message>
<xml_diff>
--- a/reports/AEGIS_LATEST.xlsx
+++ b/reports/AEGIS_LATEST.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SHREECEM (48)</t>
+          <t>SHREECEM (47)</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -700,7 +700,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-26  /  2026-06-25</t>
+          <t>2026-06-29  /  2026-06-29</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
     </row>
@@ -1568,11 +1568,11 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>8592</v>
+        <v>8717.5</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>8374 - 8810</t>
+          <t>8497 - 8938</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -1590,11 +1590,11 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+12.8%)</t>
+          <t>Above 200-DMA (+14.4%)</t>
         </is>
       </c>
       <c r="S2" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -1603,17 +1603,17 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>25776</v>
+        <v>26152</v>
       </c>
       <c r="W2" t="n">
         <v>3</v>
       </c>
       <c r="X2" t="n">
-        <v>9</v>
+        <v>10.1</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
@@ -1627,12 +1627,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — APOLLOHOSP: 78; FORTIS: 70, MAXHEALTH: 69, LALPATHLAB: 61</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — APOLLOHOSP: 78; FORTIS: 68, MAXHEALTH: 68, LALPATHLAB: 62</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Low-risk Healthcare holding (low vol) • above 200-dma (+12.8%) • outperforming Nifty • sector strength 88/100 • regime cautious (partial deploy) • 4 similar past recs: 75% positive, median +5.9%</t>
+          <t>Low-risk Healthcare holding (low vol) • above 200-dma (+14.4%) • outperforming Nifty • sector strength 88/100 • regime cautious (partial deploy) • 4 similar past recs: 75% positive, median +5.9%</t>
         </is>
       </c>
     </row>
@@ -1643,16 +1643,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Risk/Vol +25 · Historical +18 · Trend/Tech +17 · Regime +9 · Sector +3 = 72</t>
+          <t>Historical +25 · Risk/Vol +23 · Trend/Tech +13 · Regime +9 · Sector +7 = 77</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Risk/Vol</t>
+          <t>Historical</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1661,36 +1661,36 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="G3" t="n">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="H3" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="I3" t="n">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="J3" t="n">
         <v>60</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>MARICO</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>825.8</v>
+        <v>355.5</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>806 - 846</t>
+          <t>345 - 366</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -1704,15 +1704,15 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+9.0%)</t>
+          <t>Above 200-DMA (+0.0%)</t>
         </is>
       </c>
       <c r="S3" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -1721,21 +1721,21 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>23948</v>
+        <v>18133</v>
       </c>
       <c r="W3" t="n">
-        <v>29</v>
+        <v>51</v>
       </c>
       <c r="X3" t="n">
-        <v>8.1</v>
+        <v>6.1</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility FMCG name under the sector cap</t>
+          <t>Historical + Risk/Vol strongest; chosen as a lowest-volatility Power name under the sector cap</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -1745,12 +1745,12 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — MARICO: 72; NESTLEIND: 73, VBL: 61, UNITDSPR: 60. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — NTPC: 77; POWERGRID: 61, JSWENERGY: 58, NHPC: 57</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Low-risk FMCG holding (low vol) • above 200-dma (+9.0%) • sector strength 29/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +3.3%</t>
+          <t>Low-risk Power holding (low vol) • above 200-dma (+0.0%) • sector strength 71/100 • regime cautious (partial deploy) • 4 similar past recs: 100% positive, median +11.5%</t>
         </is>
       </c>
     </row>
@@ -1761,11 +1761,11 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Risk/Vol +24 · Historical +19 · Trend/Tech +15 · Regime +9 · Sector +4 = 71</t>
+          <t>Risk/Vol +25 · Historical +18 · Trend/Tech +17 · Regime +9 · Sector +3 = 72</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1779,36 +1779,36 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G4" t="n">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="H4" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="I4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="J4" t="n">
         <v>60</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>409</v>
+        <v>841.5</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>397 - 421</t>
+          <t>821 - 862</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1826,11 +1826,11 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+0.7%)</t>
+          <t>Above 200-DMA (+11.0%)</t>
         </is>
       </c>
       <c r="S4" t="n">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -1839,21 +1839,21 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>17996</v>
+        <v>25246</v>
       </c>
       <c r="W4" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="X4" t="n">
-        <v>6.1</v>
+        <v>8.6</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Financials name under the sector cap</t>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility FMCG name under the sector cap</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — KOTAKBANK: 71; ICICIBANK: 72, AXISBANK: 62, SBIN: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — MARICO: 72; NESTLEIND: 73, VBL: 61, UNITDSPR: 59. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Low-risk Financials holding (low vol) • above 200-dma (+0.7%) • outperforming Nifty • sector strength 35/100 • regime cautious (partial deploy) • 3 similar past recs: 100% positive, median +1.9%</t>
+          <t>Low-risk FMCG holding (low vol) • above 200-dma (+11.0%) • sector strength 29/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +3.3%</t>
         </is>
       </c>
     </row>
@@ -1879,76 +1879,76 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Historical +25 · Risk/Vol +23 · Regime +9 · Sector +8 · Trend/Tech +5 = 70</t>
+          <t>Risk/Vol +24 · Historical +20 · Trend/Tech +14 · Regime +9 · Sector +4 = 71</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Historical</t>
+          <t>Risk/Vol</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Trend/Tech</t>
+          <t>Sector</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="G5" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="H5" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I5" t="n">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="J5" t="n">
         <v>60</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>352</v>
+        <v>1389.7</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>342 - 363</t>
+          <t>1349 - 1430</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>+2% to +8%</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-0.9%)</t>
+          <t>Above 200-DMA (+3.3%)</t>
         </is>
       </c>
       <c r="S5" t="n">
-        <v>41</v>
+        <v>86</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -1957,21 +1957,21 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>23235</v>
+        <v>13897</v>
       </c>
       <c r="W5" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="X5" t="n">
-        <v>7.8</v>
+        <v>5</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Historical + Risk/Vol strongest; chosen as a lowest-volatility Power name under the sector cap</t>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Financials name under the sector cap</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -1981,12 +1981,12 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — NTPC: 70; POWERGRID: 62, CESC: 61, NHPC: 60</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIBANK: 71; LICI: 64, AXISBANK: 63, KOTAKBANK: 62</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Low-risk Power holding (low vol) • below 200-dma (-0.9%) • sector strength 76/100 • regime cautious (partial deploy) • 4 similar past recs: 100% positive, median +11.5%</t>
+          <t>Low-risk Financials holding (low vol) • above 200-dma (+3.3%) • sector strength 41/100 • regime cautious (partial deploy) • 8 similar past recs: 75% positive, median +5.3%</t>
         </is>
       </c>
     </row>
@@ -1997,11 +1997,11 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Risk/Vol +25 · Historical +15 · Trend/Tech +15 · Regime +9 · Sector +5 = 69</t>
+          <t>Risk/Vol +25 · Historical +15 · Trend/Tech +13 · Regime +9 · Sector +6 = 68</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2018,13 +2018,13 @@
         <v>50</v>
       </c>
       <c r="G6" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="H6" t="n">
         <v>99</v>
       </c>
       <c r="I6" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="J6" t="n">
         <v>60</v>
@@ -2040,11 +2040,11 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>2343.5</v>
+        <v>2393.1</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2284 - 2403</t>
+          <t>2332 - 2454</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -2062,11 +2062,11 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Above 200-DMA (+8.4%)</t>
+          <t>Above 200-DMA (+10.6%)</t>
         </is>
       </c>
       <c r="S6" t="n">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -2075,11 +2075,11 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>35152</v>
+        <v>35897</v>
       </c>
       <c r="W6" t="n">
         <v>15</v>
@@ -2099,12 +2099,12 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — LUPIN: 69; TORNTPHARM: 77, CIPLA: 71, ZYDUSLIFE: 71. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — LUPIN: 68; TORNTPHARM: 78, ZYDUSLIFE: 72, BIOCON: 70. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Low-risk Pharma holding (low vol) • above 200-dma (+8.4%) • sector strength 47/100 • regime cautious (partial deploy) • no historical analogue yet (&lt;3 obs)</t>
+          <t>Low-risk Pharma holding (low vol) • above 200-dma (+10.6%) • sector strength 59/100 • regime cautious (partial deploy) • no historical analogue yet (&lt;3 obs)</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Risk/Vol +24 · Historical +23 · Regime +9 · Trend/Tech +6 · Sector +4 = 66</t>
+          <t>Risk/Vol +24 · Historical +21 · Regime +9 · Trend/Tech +6 · Sector +6 = 66</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2133,58 +2133,58 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G7" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H7" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I7" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="J7" t="n">
         <v>60</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>ABBOTINDIA</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>1850.7</v>
+        <v>25675</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>1801 - 1900</t>
+          <t>24956 - 26394</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>-3% to +15%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-5.2%)</t>
+          <t>Below 200-DMA (-7.9%)</t>
         </is>
       </c>
       <c r="S7" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -2193,21 +2193,21 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V7" t="n">
-        <v>20358</v>
+        <v>25675</v>
       </c>
       <c r="W7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>7.1</v>
+        <v>12.7</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Telecom name under the sector cap</t>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Pharma name under the sector cap</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -2217,27 +2217,27 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BHARTIARTL: 66; TATACOMM: 53, INDUSTOWER: 50</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ABBOTINDIA: 66; TORNTPHARM: 78, ZYDUSLIFE: 72, BIOCON: 70. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>Low-risk Telecom holding (low vol) • below 200-dma (-5.2%) • sector strength 41/100 • regime cautious (partial deploy) • 13 similar past recs: 69% positive, median +12.5%</t>
+          <t>Low-risk Pharma holding (low vol) • below 200-dma (-7.9%) • sector strength 59/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +24.6%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BUY</t>
+          <t>STRONG BUY</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Risk/Vol +24 · Historical +21 · Regime +9 · Trend/Tech +5 · Sector +5 = 64</t>
+          <t>Risk/Vol +24 · Historical +23 · Regime +9 · Trend/Tech +6 · Sector +4 = 66</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2251,58 +2251,58 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="G8" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="H8" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I8" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="J8" t="n">
         <v>60</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Pharma</t>
+          <t>Telecom</t>
         </is>
       </c>
       <c r="M8" t="n">
-        <v>25585</v>
+        <v>1845</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>24868 - 26302</t>
+          <t>1796 - 1894</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-3% to +15%</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-8.3%)</t>
+          <t>Below 200-DMA (-5.5%)</t>
         </is>
       </c>
       <c r="S8" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -2311,21 +2311,21 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>25585</v>
+        <v>33210</v>
       </c>
       <c r="W8" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="X8" t="n">
-        <v>11.6</v>
+        <v>11.4</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Pharma name under the sector cap</t>
+          <t>Risk/Vol + Historical strongest; chosen as a lowest-volatility Telecom name under the sector cap</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -2335,12 +2335,12 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ABBOTINDIA: 64; TORNTPHARM: 77, CIPLA: 71, ZYDUSLIFE: 71. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — BHARTIARTL: 66; TATACOMM: 53, INDUSTOWER: 51</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Low-risk Pharma holding (low vol) • below 200-dma (-8.3%) • sector strength 47/100 • regime cautious (partial deploy) • 2 similar past recs: 100% positive, median +24.6%</t>
+          <t>Low-risk Telecom holding (low vol) • below 200-dma (-5.5%) • sector strength 35/100 • regime cautious (partial deploy) • 13 similar past recs: 69% positive, median +12.5%</t>
         </is>
       </c>
     </row>
@@ -2351,11 +2351,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Risk/Vol +23 · Historical +17 · Regime +9 · Sector +8 · Trend/Tech +5 = 62</t>
+          <t>Risk/Vol +23 · Historical +17 · Regime +9 · Sector +7 · Trend/Tech +5 = 61</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2372,13 +2372,13 @@
         <v>56</v>
       </c>
       <c r="G9" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H9" t="n">
         <v>92</v>
       </c>
       <c r="I9" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="J9" t="n">
         <v>60</v>
@@ -2394,11 +2394,11 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>283.9</v>
+        <v>285.5</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>275 - 293</t>
+          <t>277 - 294</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -2412,15 +2412,15 @@
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-0.8%)</t>
+          <t>Below 200-DMA (-0.2%)</t>
         </is>
       </c>
       <c r="S9" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -2429,17 +2429,17 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V9" t="n">
-        <v>19305</v>
+        <v>17130</v>
       </c>
       <c r="W9" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -2453,12 +2453,12 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — POWERGRID: 62; NTPC: 70, CESC: 61, NHPC: 60. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — POWERGRID: 61; NTPC: 77, JSWENERGY: 58, NHPC: 57. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>Low-risk Power holding (low vol) • below 200-dma (-0.8%) • sector strength 76/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +12.3%</t>
+          <t>Low-risk Power holding (low vol) • below 200-dma (-0.2%) • sector strength 71/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +12.3%</t>
         </is>
       </c>
     </row>
@@ -2490,13 +2490,13 @@
         <v>52</v>
       </c>
       <c r="G10" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H10" t="n">
         <v>96</v>
       </c>
       <c r="I10" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="J10" t="n">
         <v>60</v>
@@ -2512,11 +2512,11 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>1813.6</v>
+        <v>1799</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>1763 - 1865</t>
+          <t>1748 - 1850</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-3.6%)</t>
+          <t>Below 200-DMA (-4.3%)</t>
         </is>
       </c>
       <c r="S10" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -2547,17 +2547,17 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>27204</v>
+        <v>17990</v>
       </c>
       <c r="W10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="X10" t="n">
-        <v>9.1</v>
+        <v>6.5</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -2571,12 +2571,12 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIGI: 60; ICICIBANK: 72, KOTAKBANK: 71, AXISBANK: 62. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — ICICIGI: 60; ICICIBANK: 71, LICI: 64, AXISBANK: 63. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Low-risk Financials holding (low vol) • below 200-dma (-3.6%) • sector strength 35/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +7.7%</t>
+          <t>Low-risk Financials holding (low vol) • below 200-dma (-4.3%) • sector strength 41/100 • regime cautious (partial deploy) • 2 similar past recs: 50% positive, median +7.7%</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2591,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Risk/Vol +22 · Historical +17 · Regime +9 · Trend/Tech +5 · Sector +1 = 54</t>
+          <t>Risk/Vol +22 · Historical +17 · Regime +9 · Trend/Tech +4 · Sector +2 = 54</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2608,13 +2608,13 @@
         <v>56</v>
       </c>
       <c r="G11" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="H11" t="n">
         <v>90</v>
       </c>
       <c r="I11" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="J11" t="n">
         <v>60</v>
@@ -2630,11 +2630,11 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>1318.1</v>
+        <v>1309.9</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>1276 - 1360</t>
+          <t>1269 - 1351</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -2652,11 +2652,11 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-7.2%)</t>
+          <t>Below 200-DMA (-7.8%)</t>
         </is>
       </c>
       <c r="S11" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -2665,17 +2665,17 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>25044</v>
+        <v>24888</v>
       </c>
       <c r="W11" t="n">
         <v>19</v>
       </c>
       <c r="X11" t="n">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
@@ -2689,12 +2689,12 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — RELIANCE: 54; GAIL: 59, IGL: 51, PETRONET: 50. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — RELIANCE: 54; GAIL: 60, IGL: 52, PETRONET: 52. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>Low-risk Energy holding (low vol) • below 200-dma (-7.2%) • sector strength 12/100 • regime cautious (partial deploy) • 8 similar past recs: 62% positive, median +4.3%</t>
+          <t>Low-risk Energy holding (low vol) • below 200-dma (-7.8%) • sector strength 18/100 • regime cautious (partial deploy) • 8 similar past recs: 62% positive, median +4.3%</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2726,7 @@
         <v>32</v>
       </c>
       <c r="G12" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H12" t="n">
         <v>98</v>
@@ -2748,11 +2748,11 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>5237</v>
+        <v>5229</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>5099 - 5375</t>
+          <t>5091 - 5367</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -2770,11 +2770,11 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-9.6%)</t>
+          <t>Below 200-DMA (-9.7%)</t>
         </is>
       </c>
       <c r="S12" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -2783,17 +2783,17 @@
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>15711</v>
+        <v>26145</v>
       </c>
       <c r="W12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="X12" t="n">
-        <v>7</v>
+        <v>8.9</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>Low-risk FMCG holding (low vol) • below 200-dma (-9.6%) • sector strength 29/100 • regime cautious (partial deploy) • 3 similar past recs: 33% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
+          <t>Low-risk FMCG holding (low vol) • below 200-dma (-9.7%) • sector strength 29/100 • regime cautious (partial deploy) • 3 similar past recs: 33% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
         </is>
       </c>
     </row>
@@ -2823,11 +2823,11 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Risk/Vol +22 · Regime +9 · Trend/Tech +8 · Historical +7 · Sector +2 = 48</t>
+          <t>Risk/Vol +23 · Regime +9 · Historical +7 · Trend/Tech +6 · Sector +2 = 47</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2844,13 +2844,13 @@
         <v>24</v>
       </c>
       <c r="G13" t="n">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="H13" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I13" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="J13" t="n">
         <v>60</v>
@@ -2866,11 +2866,11 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>25735</v>
+        <v>25600</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>24925 - 26545</t>
+          <t>24794 - 26406</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -2884,15 +2884,15 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Below 200-DMA (-2.7%)</t>
+          <t>Below 200-DMA (-3.1%)</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V13" t="n">
@@ -2911,7 +2911,7 @@
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>7.1</v>
+        <v>4.4</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
@@ -2925,12 +2925,12 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — SHREECEM: 48; GRASIM: 75, ULTRACEMCO: 57, RAMCOCEM: 48. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
+          <t>Picked by lowest-vol + sector cap (the validated rule). Evidence scores — SHREECEM: 47; GRASIM: 75, ULTRACEMCO: 56, RAMCOCEM: 49. Note: a peer scores higher but is higher-vol or cap-excluded — Evidence Score is context, not the selector.</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>Low-risk Cement holding (low vol) • below 200-dma (-2.7%) • sector strength 18/100 • regime cautious (partial deploy) • 5 similar past recs: 40% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
+          <t>Low-risk Cement holding (low vol) • below 200-dma (-3.1%) • sector strength 24/100 • regime cautious (partial deploy) • 5 similar past recs: 40% positive, median -7.7% • HELD FOR DIVERSIFICATION despite weak historical analogue — sized by risk, not conviction</t>
         </is>
       </c>
     </row>
@@ -27719,7 +27719,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>14.9%</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -27729,12 +27729,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>FMCG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9.1%</t>
+          <t>10.5%</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -27744,12 +27744,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FMCG</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>9.0%</t>
+          <t>7.1%</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -27759,12 +27759,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Power</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>6.9%</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -27774,12 +27774,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Telecom</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>5.4%</t>
+          <t>6.8%</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -27789,12 +27789,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5.0%</t>
+          <t>6.1%</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -27804,12 +27804,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cement</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>5.0%</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -27819,12 +27819,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>Cement</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4.3%</t>
+          <t>2.7%</t>
         </is>
       </c>
       <c r="C9" t="n">

</xml_diff>